<commit_message>
Method 1 (Rappler Done), TODO: Youtube.,
</commit_message>
<xml_diff>
--- a/Social Computing/rappler.xlsx
+++ b/Social Computing/rappler.xlsx
@@ -456,33 +456,40 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FACT CHECK: VP Sara Duterte's face is in her book 'Isang Kaibigan'</t>
+          <t>Accenture’s sustainability value promise</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.rappler.com/newsbreak/fact-check/sara-duterte-face-book-isang-kaibigan/</t>
+          <t>https://www.rappler.com/brandrap/accenture-philippines-sustainability-value-promise</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2024-08-22T20:11:07+08:00</t>
+          <t>2022-05-02T17:00:00+08:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Claim: The face of Vice President Sara Duterte is not in the children’s book that she wrote titled, “Isang Kaibigan“.
-Why we fact-checked this: The claim can be found in an August 21 post on social media platform X (formerly Twitter). The post says: “Yung libro na ni anino ni VPISD eh wala nga dyan” (The book that does not bear even a hint of a shadow of VPISD [Vice President Inday Sara Duterte] is not there).
-The post also includes a video from the TikTok account “klc4.0” which — referring to Duterte’s book, Isang Kaibigan — says: “Yung libro ni Sara Duterte na walang mukha niya” (The book of Sara Duterte that does not carry her face).
-As of writing, the post on X already has around 51 comments, 50 shares, 135 reactions, 7 bookmarks, and 23,800 video views. The source video on TikTok, meanwhile, has around 198,700 views, 3,690 reactions, 1,076 comments, 226 bookmarks, and 138 shares. 
-Both the X post and the TikTok video compare Sara Duterte and Senator Risa Hontiveros, pointing out the supposed absence of Duterte’s face in her book unlike Hontiveros whose face is supposedly on billboards and buses.
-The facts: Vice President Sara Duterte’s book, “Isang Kaibigan” actually shows her face at the end of the book. 
-Numerous news reports have shown the page of the book that contains Duterte’s picture, along with some biographical details and the statement, “Siya ay isang tunay na kaibigan” (She is a true friend). Examples are news articles published on August 21 by Rappler, Philstar.com, and Inquirer.net.
-What’s the issue: The controversy over the book arose during the August 20 budget hearing for the Office of the Vice President’s (OVP) proposed 2025 budget. Senator Hontiveros asked Duterte about the book for which the OVP allotted a P10-million budget for printing and distribution. 
-Duterte, however, replied, accusing Hontiveros of “politicizing the budget hearing.” This did not sit well with senator, who later on told Duterte: “Budget hearing po ito. Hindi po lahat about you. Pera po ito ng taong bayan.” (This is a budget hearing. Not everything is about you. This is about public funds.) (READ: Rappler Recap: Sara Duterte, Risa Hontiveros clash during Senate budget hearing)
-Duterte’s book is about an owl (Kwago) with many friends. A storm damaged the owl’s home; with the others gone, one of the owl’s friends, a parrot (Loro), offered to help the owl recover from the storm’s effects. – Percival Bueser/ Rappler.com 
-Percival Bueser is a graduate of Rappler’s fact-checking mentorship program. This fact check was reviewed by a member of Rappler’s research team and a senior editor. Learn more about Rappler’s fact-checking mentorship program here.
-Keep us aware of suspicious Facebook pages, groups, accounts, websites, articles, or photos in your network by contacting us at factcheck@rappler.com. You may also report dubious claims to #FactsFirstPH tipline by messaging Rappler on Facebook or Newsbreak via Twitter direct message. You may also report through our Viber fact check chatbot. Let us battle disinformation one Fact Check at a time.
+          <t xml:space="preserve">Editor’s note: This content is sponsored by Accenture and was produced by BrandRap, the sales and marketing arm of Rappler. No member of the news and editorial team participated in the production of this piece. This article was written with Accenture.
+When we think of sustainability, we often picture the environment or equate it to green practices.
+However, sustainability spans environmental, social, and governance (ESG) issues, from transitioning to a zero-carbon economy to human rights to inclusion and diversity. Accenture, together with its partners, is helping to solve these to achieve the United Nations Sustainable Development Goals. 
+Following Accenture’s global sustainability agenda, Accenture in the Philippines continues its efforts by operating as a responsible company, client partner, and citizen with the goal of creating value for its people, clients, and the community. 
+According to their United Nations Global Compact: Communication on Progress 2021, they have identified eight high and four secondary priority UN Sustainable Development Goals where Accenture operations will have the most impact. With this, Accenture in the Philippines is working on four key focus areas: caring for their people and accelerating equality, caring for communities, readying the path to net-zero by 2025, and practicing technology sustainability. 
+Accenture in the Philippines continues to put its people’s safety and health, learning, growth, and well-being as a priority. Strongly committed to inclusion and diversity in its organization, they continue to build diverse teams made up of individuals that are empowered to be their true selves and utilize their different talents in creating innovative solutions. 
+They are accelerating gender equality, supporting the LGBT+ community, strengthening disability inclusion and boosting accessibility, and promoting the value of cross-cultural diversity. They do this via bold leadership – where leaders set targets for inclusion and diversity and walk the talk, comprehensive action – wherein policies and practices are put in place to ensure that a culture of equality is consistently exhibited and respected, and empowering environment – where people and communities are encouraged and enabled every time to thrive and succeed.
+Accenture continues to strengthen communities by making a difference and creating shared success to build a more inclusive and equitable future. Through innovations and partnerships, they aim to help alleviate poverty and hunger, provide livelihood, tech-vocational and entrepreneurial training, upskill individuals and give access to education, help in disaster recovery, and mitigate the COVID-19 impact on the country. 
+Examples of the work include:
+The pandemic may have shifted a lot of the volunteering initiatives into virtual events, but Accenture’s passionate volunteers showed greater enthusiasm than before to help address societal issues. 
+They participated in various digital platforms that either teach one how to code (Hour of Code), create an accessible map of an area that has humanitarian needs (Missing Maps), or participate in real scientific research (Zooniverse) that contributes to a better and more sustainable world.
+Its Skills to Succeed Academy helps fellow Filipinos plan and prepare for a successful career journey by equipping them with employability skills that will enable them to be future-ready. 
+Supported by Skills to Succeed, their Near-Hire Training (NHT) program aims to develop the right job skills for individuals from poor communities, helping them become competitive and marketable. They have had more than 1,300 beneficiaries in the last five years of which 193 NHT trainees were hired in Accenture in the Philippines.
+Their people’s donations also helped the charitable programs that span from helping provide PPEs to frontliners and medical equipment to various hospitals and health centers, providing equipment to selected public schools, supporting Accenture custodians and security personnel, and mobilizing disaster relief packs for calamity-stricken individuals and communities. 
+Accenture has committed to reaching net-zero carbon emissions by 2025. To do this, they will: 
+With their years of investment and experience, they have developed a suite of Sustainability Services to help their clients become more sustainable and competitive. 
+Accenture has made sustainability one of their greatest responsibilities, and with everyone understanding that every action has an impact, it can be the force of change the world needs right now. 
+To learn more about Accenture’s sustainability commitments, head over to the website. – Rappler.com
+*Key suppliers are defined as vendors that represent a significant portion of Accenture’s 2019 Scope 3 emissions.
 </t>
         </is>
       </c>

</xml_diff>

<commit_message>
Revised Method : Youtube
</commit_message>
<xml_diff>
--- a/Social Computing/rappler.xlsx
+++ b/Social Computing/rappler.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>